<commit_message>
refactor: remove campo Tipo de Pagamento da importação Excel
- payment_type derivado automaticamente: convenio preenchido → 'convenio',
  caso contrário → 'particular'
- Coluna removida de PlanilhaRow, COLUMN_MAP, prévia e planilha modelo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelo-pacientes.xlsx
+++ b/public/modelo-pacientes.xlsx
@@ -397,20 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,59 +439,21 @@
         <v>Clínica</v>
       </c>
       <c r="I1" t="str">
-        <v>Tipo de Pagamento</v>
+        <v>Valor por Sessão</v>
       </c>
       <c r="J1" t="str">
-        <v>Valor por Sessão</v>
+        <v>Convênio</v>
       </c>
       <c r="K1" t="str">
-        <v>Convênio</v>
+        <v>CPF</v>
       </c>
       <c r="L1" t="str">
         <v>Observações</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Maria Silva Santos</v>
-      </c>
-      <c r="B2" t="str">
-        <v>12/05/2015</v>
-      </c>
-      <c r="C2" t="str">
-        <v>TEA - Transtorno do Espectro Autista</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ana Paula Santos</v>
-      </c>
-      <c r="E2" t="str">
-        <v>(11) 98765-4321</v>
-      </c>
-      <c r="F2" t="str">
-        <v>ana.santos@email.com</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Mãe</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Clínica Girassol</v>
-      </c>
-      <c r="I2" t="str">
-        <v>particular</v>
-      </c>
-      <c r="J2" t="str">
-        <v>150,00</v>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
-        <v>Paciente com boa evolução nas sessões de ABA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>